<commit_message>
criteria extraction done, analysis is ongoing
</commit_message>
<xml_diff>
--- a/coding/criteria extraction/Amelia/Amelia_coding-sheet_criteria_extraction.xlsx
+++ b/coding/criteria extraction/Amelia/Amelia_coding-sheet_criteria_extraction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\01 DE\5. postdoc\SocEnRep Project\WP1 &amp; 2\litsearch\coding\criteria extraction\Amelia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD23CE4-F8A7-479D-8449-28FF87D7A00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEE5FC9-9E63-4928-ACBB-4AED2E5DE11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4339,7 +4339,7 @@
     <t>Set up the reproduction package using version control software, such as Git.</t>
   </si>
   <si>
-    <t>code documentation/anotation</t>
+    <t>code documentation/annotation</t>
   </si>
   <si>
     <t>code documentation/annotation</t>
@@ -4519,7 +4519,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4546,6 +4546,9 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4559,12 +4562,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4900,11 +4897,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
     </row>
     <row r="2" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -4912,11 +4909,11 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
     </row>
     <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -4930,18 +4927,18 @@
       <c r="A5" s="5"/>
     </row>
     <row r="7" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
     </row>
     <row r="8" spans="1:3" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
     </row>
     <row r="10" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -4999,25 +4996,25 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
     </row>
     <row r="17" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
     </row>
     <row r="19" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
     </row>
     <row r="20" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
@@ -5174,11 +5171,11 @@
       </c>
     </row>
     <row r="35" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
     </row>
     <row r="36" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
@@ -5236,11 +5233,11 @@
       </c>
     </row>
     <row r="42" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="10" t="s">
+      <c r="A42" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
     </row>
     <row r="43" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
@@ -5276,18 +5273,18 @@
       </c>
     </row>
     <row r="47" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
     </row>
     <row r="48" spans="1:3" ht="135.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="14" t="s">
+      <c r="A48" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -12205,7 +12202,7 @@
       <c r="F3" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="7" t="s">
         <v>921</v>
       </c>
       <c r="H3" s="7" t="s">
@@ -12234,7 +12231,7 @@
       <c r="F4" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="7" t="s">
         <v>921</v>
       </c>
       <c r="H4" s="7" t="s">
@@ -12307,7 +12304,7 @@
         <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
         <v>49</v>
@@ -12376,7 +12373,7 @@
       <c r="F9" t="s">
         <v>61</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="10" t="s">
         <v>930</v>
       </c>
       <c r="H9" s="7" t="s">
@@ -12405,7 +12402,7 @@
       <c r="F10" t="s">
         <v>61</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="10" t="s">
         <v>930</v>
       </c>
       <c r="H10" s="7" t="s">
@@ -12434,7 +12431,7 @@
       <c r="F11" t="s">
         <v>61</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="10" t="s">
         <v>928</v>
       </c>
       <c r="H11" s="7" t="s">
@@ -12463,7 +12460,7 @@
       <c r="F12" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="10" t="s">
         <v>929</v>
       </c>
       <c r="H12" s="7" t="s">
@@ -12495,7 +12492,7 @@
       <c r="F13" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="10" t="s">
         <v>924</v>
       </c>
       <c r="J13" s="7"/>

</xml_diff>